<commit_message>
Reword first three Time Log entries; correct transaction count to ~64k
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Methodology.xlsx
+++ b/Methodology.xlsx
@@ -549,7 +549,7 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>I started from the questions, not the data. I wrote down the 10 business questions I wanted to answer first (price changes, a competitor in the East, the cost of stockouts, and so on). The first batch of data was too flat to answer them, so I asked for more realistic numbers with real patterns. That grew the transactions to about 60k rows and added the extra files — marketing, promotions, stockouts, competitor activity, weather, market size — so each question could actually be answered.</t>
+          <t>I started from the questions. I wrote down a few business questions I wanted to answer (price changes, a competitor in the East, the cost of stockouts, and so on). The first batch of data was too flat to answer them, so I asked for more realistic numbers with real patterns. That grew the transactions to about 64k rows and added the extra files — marketing, promotions, stockouts, competitor activity, weather, market size — so each question could actually be answered.</t>
         </is>
       </c>
     </row>
@@ -576,7 +576,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>I tightened the cleaning rules (handling duplicate rows and messy formats) and decided myself how the monthly table should be shaped — one row per month, category and region.</t>
+          <t>Tightened the cleaning rules (handling duplicate rows and messy formats) and decided how the monthly table should be shaped — one row per month, category and region.</t>
         </is>
       </c>
     </row>
@@ -603,7 +603,7 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>I set one firm rule: Claude only ever sees summary numbers, never the real revenue. I also kept the model simple (Ridge) instead of something heavier — see the Decision Log.</t>
+          <t>Set one firm rule: Claude only ever sees summary numbers, never the real revenue. I also kept the model simple (Ridge) instead of something heavier — see the Decision Log.</t>
         </is>
       </c>
     </row>

</xml_diff>